<commit_message>
Added charts & improved client output
</commit_message>
<xml_diff>
--- a/results/articles.xlsx
+++ b/results/articles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,36 +499,74 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>cybersecurity in Modern Systems</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Maria Lopez, David Wilson</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>10.1000/xyz456</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>This paper analyzes the role of cybersecurity in modern systems.</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Lopez, M., &amp; Wilson, D. (2023). cybersecurity in Modern Systems. International Journal of Security Studies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Challenges of cybersecurity</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Emily Johnson, Robert White</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="C4" t="n">
         <v>2020</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>10.1000/xyz789</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>This article explores the main challenges of cybersecurity.</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="F4" t="n">
         <v>27</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Johnson, E., &amp; White, R. (2020). Challenges of cybersecurity. European Security Review.</t>
         </is>

</xml_diff>

<commit_message>
improved charts an design
</commit_message>
<xml_diff>
--- a/results/articles.xlsx
+++ b/results/articles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,12 +461,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Recent Advances in cybersecurity</t>
+          <t>Secure Communication Protocols in Distributed Networks</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>John Smith, Anna Brown</t>
+          <t>Carlos Ruiz, Emma Scott</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -474,101 +474,63 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.1000/xyz123</t>
+          <t>10.1000/xyz102</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>This article discusses recent advances in cybersecurity.</t>
+          <t>This article reviews secure communication protocols used in distributed networks.</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Smith, J., &amp; Brown, A. (2021). Recent Advances in cybersecurity. Journal of Network Research.</t>
+          <t>Ruiz, C., &amp; Scott, E. (2021). Secure Communication Protocols in Distributed Networks. Journal of Communication Security.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cybersecurity in Modern Systems</t>
+          <t>Secure Network Architectures for Smart Cities</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Maria Lopez, David Wilson</t>
+          <t>Helen Young, James Harris</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.1000/xyz456</t>
+          <t>10.1000/xyz106</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>This paper analyzes the role of cybersecurity in modern systems.</t>
+          <t>This article presents secure network architectures for smart cities.</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Lopez, M., &amp; Wilson, D. (2023). cybersecurity in Modern Systems. International Journal of Security Studies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Challenges of cybersecurity</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Emily Johnson, Robert White</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>10.1000/xyz789</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>This article explores the main challenges of cybersecurity.</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>27</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Johnson, E., &amp; White, R. (2020). Challenges of cybersecurity. European Security Review.</t>
+          <t>Young, H., &amp; Harris, J. (2021). Secure Network Architectures for Smart Cities. Smart Infrastructure Review.</t>
         </is>
       </c>
     </row>

</xml_diff>